<commit_message>
Updated check.xlsx with latest changes
</commit_message>
<xml_diff>
--- a/check.xlsx
+++ b/check.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshi\Downloads\test excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{728A5F78-6A11-4FB1-A259-B31D1C134C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{015A323D-2CE6-4CB5-A59B-C61B566F40F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{60E4E408-3CD0-4601-AE7F-E88ED1D4FAD1}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>column1</t>
   </si>
@@ -34,6 +34,12 @@
   </si>
   <si>
     <t>column3</t>
+  </si>
+  <si>
+    <t>column4</t>
+  </si>
+  <si>
+    <t>column5</t>
   </si>
 </sst>
 </file>
@@ -405,10 +411,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD129880-A1E4-4004-B325-A11C62CE00DD}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -418,6 +424,12 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>